<commit_message>
Profiling 07: the adviser's reported LEI is lookup only (operator ruling)
Advisers report an affiliate's or another firm's LEI in Form ADV Item 1.P
(8 valid LEIs on 2 to 7 advisers each over 13 months), so the full run
stopped on an identifier conflict. Operator, 2026-10-09: "Keep LEI, lookup
only (Recommended)". The filings contract keeps it as cross-reference
reported_lei; CRD alone is the adviser's identity. The LEI Identifier
Contract lists custodians only. Form ADV policy digest af0fa7cc...

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFKdv4nqKXKM9d5Cf2hEFk
</commit_message>
<xml_diff>
--- a/rules/sources/iapd.adv/MAPPING.xlsx
+++ b/rules/sources/iapd.adv/MAPPING.xlsx
@@ -1036,7 +1036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1121,7 +1121,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.filings.v1</t>
+          <t>iapd.adv.custodians.v1</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>No: lookup only</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>mdm.iapd.adv.filings.v1.contract.adapter.identifiers.lei</t>
+          <t>mdm.iapd.adv.custodians.v1.contract.adapter.identifiers.lei</t>
         </is>
       </c>
     </row>
@@ -1163,19 +1163,15 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>lei</t>
+          <t>bd_number</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>lei</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>lei</t>
-        </is>
-      </c>
+          <t>bd_number</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1187,39 +1183,6 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>mdm.iapd.adv.custodians.v1.contract.adapter.identifiers.lei</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>iapd.adv.custodians.v1</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>bd_number</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>bd_number</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Only with a new dataset code</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>mdm.iapd.adv.custodians.v1.contract.adapter.identifiers.bd_number</t>
         </is>

</xml_diff>

<commit_message>
Profiling 07: a custodian is named by its BD number first (operator ruling)
Advisers report the right broker-dealer number but often a parent's or
another LEI (8 BD numbers with 2 to 4 valid LEIs each), so the second full
run stopped on an identifier conflict among custodians. Operator,
2026-10-09: "BD number first (Recommended)". custodian_id is bd:, else
lei:, else name:; the LEI identifies a custodian only when its row has no BD
number; every reported LEI is kept as cross-reference reported_lei.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFKdv4nqKXKM9d5Cf2hEFk
</commit_message>
<xml_diff>
--- a/rules/sources/iapd.adv/MAPPING.xlsx
+++ b/rules/sources/iapd.adv/MAPPING.xlsx
@@ -1041,7 +1041,7 @@
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
@@ -1126,19 +1126,15 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>lei</t>
+          <t>bd_number</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>lei</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>lei</t>
-        </is>
-      </c>
+          <t>bd_number</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1151,7 +1147,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>mdm.iapd.adv.custodians.v1.contract.adapter.identifiers.lei</t>
+          <t>mdm.iapd.adv.custodians.v1.contract.adapter.identifiers.bd_number</t>
         </is>
       </c>
     </row>
@@ -1163,15 +1159,19 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>bd_number</t>
+          <t>lei</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>bd_number</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
+          <t>custodian_lei</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>lei</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>mdm.iapd.adv.custodians.v1.contract.adapter.identifiers.bd_number</t>
+          <t>mdm.iapd.adv.custodians.v1.contract.adapter.identifiers.lei</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ticket 75: an adviser links to its custodians (CUSTODIAN)
combine.yaml collects each filing's distinct custodian ids from its custody
rows; the filings contract links the adviser to the custodians contract's
record of each in the same monthly file. CUSTODIAN is back in the
relationship types (v4) and the context definitions; the policy's pinned
layer chain gains it as one layer, and the integration answer file's policy
digest moves. Configuration only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199JiQoZJ5my5vrS5tW3FQH
</commit_message>
<xml_diff>
--- a/rules/sources/iapd.adv/MAPPING.xlsx
+++ b/rules/sources/iapd.adv/MAPPING.xlsx
@@ -638,14 +638,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -904,60 +904,64 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.custodians.v1</t>
+          <t>iapd.adv.filings.v1</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr"/>
+          <t>relationship CUSTODIAN</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>legal_name</t>
+          <t>published, item</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>MDM field</t>
+          <t>Link to iapd.adv.custodians.v1</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>mdm.iapd.adv.custodians.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.name</t>
+          <t>mdm.iapd.adv.filings.v1.contract.adapter.relationships</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.custodians.v1</t>
+          <t>iapd.adv.filings.v1</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>address</t>
+          <t>relationship CUSTODIAN</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>each</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>custodians</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>MDM field</t>
+          <t>One link per item (item.)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>mdm.iapd.adv.custodians.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.address</t>
+          <t>mdm.iapd.adv.filings.v1.contract.adapter.relationships</t>
         </is>
       </c>
     </row>
@@ -969,17 +973,13 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>address</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>legal_name</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>mdm.iapd.adv.custodians.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.address</t>
+          <t>mdm.iapd.adv.custodians.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.name</t>
         </is>
       </c>
     </row>
@@ -1006,20 +1006,84 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>MDM field</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>mdm.iapd.adv.custodians.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.address</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>iapd.adv.custodians.v1</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>address</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>MDM field</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>mdm.iapd.adv.custodians.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.address</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>iapd.adv.custodians.v1</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>address</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
           <t>country</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>country</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>MDM field</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>mdm.iapd.adv.custodians.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.address</t>
         </is>

</xml_diff>

<commit_message>
Ticket 129, fix 5: a custodian's record key is the custodian alone
Operator: "Fix 5". iapd.adv.custodians.v1 keys on custodian_id; the month is
the publication's (publication_key per file, revision YYYYMM, effective_at the
month end), so each month restates one record. The CUSTODIAN link targets
[item]. The data-onboarding skill records the record-key rule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YGQ3FjYgHS7jgMe6eLB7Z3
</commit_message>
<xml_diff>
--- a/rules/sources/iapd.adv/MAPPING.xlsx
+++ b/rules/sources/iapd.adv/MAPPING.xlsx
@@ -587,7 +587,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>one custodian named in one monthly file (the file's month end and custodian_id, from its first custody row in the file); a custodian's records join by LEI or SEC broker-dealer number</t>
+          <t>one custodian (custodian_id, from its first custody row in a file); each monthly file restates it as a new publication; a custodian's records join by LEI or SEC broker-dealer number</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
@@ -919,7 +919,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>published, item</t>
+          <t>item</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">

</xml_diff>